<commit_message>
Les questions bonus (travail en cours)
</commit_message>
<xml_diff>
--- a/contenu/sanctuaire-cahier-de-contenu.xlsx
+++ b/contenu/sanctuaire-cahier-de-contenu.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Parcours" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Textes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Quiz" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pop quiz" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -693,13 +694,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="105" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="21" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -714,6 +716,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -735,10 +738,11 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>LES QUATRE ONGLETS, EN BAS DE L'ECRAN</t>
+          <t>LES CINQ ONGLETS, EN BAS DE L'ECRAN</t>
         </is>
       </c>
     </row>
@@ -770,88 +774,98 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="3" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Pop quiz      ....  les questions bonus qui surgissent sans QR code pendant le parcours</t>
+        </is>
+      </c>
+    </row>
+    <row r="15"/>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>CE QUE TU DOIS REMPLIR</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="5" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">     Les cases sur fond creme sont a remplir par toi.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="6" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">     Les cases sur fond gris sont calculees ou fixees, tu peux les ignorer.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="7" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">     Les cases sur fond rose sont des questions qui attendent ta reponse.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>AVANCEMENT</t>
-        </is>
-      </c>
-    </row>
+    <row r="20"/>
     <row r="21" ht="45" customHeight="1">
       <c r="B21" s="3" t="inlineStr">
         <is>
+          <t>AVANCEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
           <t>86 textes a ecrire au total, repartis sur les 17 etapes.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="8" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Astuce pour suivre ton avancement : clique sur la lettre F en haut de la colonne des textes, dans l'onglet Textes. En bas a droite de l'ecran, Excel affiche le nombre de cases remplies.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="75" customHeight="1">
-      <c r="B24" s="3" t="inlineStr">
+    <row r="24" ht="75" customHeight="1"/>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>QUATRE QUESTIONS AVANT QUE JE FABRIQUE QUOI QUE CE SOIT</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="13" t="inlineStr">
+    <row r="26" ht="60" customHeight="1">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">1. COMBIEN DE QR CODES ? </t>
         </is>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1"/>
-    <row r="27">
-      <c r="B27" s="9" t="inlineStr">
+    <row r="27"/>
+    <row r="28" ht="45" customHeight="1">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>2. LES LETTRES DE L'ENIGME. En sens B, le joueur ramasse I, R, I, S dans cet ordre : le mot est deja ecrit, l'enigme du Jardin des Iris se resout sans reflechir. En sens A il ramasse R, I, S, I et doit chercher. Veux-tu permuter deux lettres pour reequilibrer ?</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="45" customHeight="1"/>
-    <row r="29">
-      <c r="B29" s="9" t="inlineStr">
+    <row r="29"/>
+    <row r="30" ht="75" customHeight="1">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>3. LE CODE DE LA SERRE. Le joueur tape-t-il IRIS sur le site, ou sur un cadenas physique ? Si c'est sur le site, c'est une mecanique a construire, dis-le moi.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="75" customHeight="1"/>
-    <row r="31">
-      <c r="B31" s="9" t="inlineStr">
+    <row r="31"/>
+    <row r="32">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>4. LES DEUX PISTES DE LA COLLEGUE SOIGNEUSE. Sur ton schema, elle ouvre deux branches : les cameras puis le plan d'un cote, les jumelles puis l'enclos des loups de l'autre. Les deux sont-elles obligatoires, ou la premiere est-elle facultative ? J'ai suppose qu'on les fait l'une apres l'autre.</t>
         </is>
@@ -4379,4 +4393,292 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="56" customHeight="1">
+      <c r="A1" s="50" t="inlineStr">
+        <is>
+          <t>LES QUESTIONS BONUS. Elles surgissent sans QR code, pendant le parcours. Une seule tentative : qui répond juste du premier coup gagne un indice que les autres n'auront pas. « Moment » vaut « au scan » (dès l'ouverture de la borne) ou « avant la sortie » (juste avant l'écran qui indique où aller). Une proposition laissée vide est ignorée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="51" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B2" s="51" t="inlineStr">
+        <is>
+          <t>Moment</t>
+        </is>
+      </c>
+      <c r="C2" s="51" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="D2" s="51" t="inlineStr">
+        <is>
+          <t>Proposition 1</t>
+        </is>
+      </c>
+      <c r="E2" s="51" t="inlineStr">
+        <is>
+          <t>Proposition 2</t>
+        </is>
+      </c>
+      <c r="F2" s="51" t="inlineStr">
+        <is>
+          <t>Proposition 3</t>
+        </is>
+      </c>
+      <c r="G2" s="51" t="inlineStr">
+        <is>
+          <t>Proposition 4</t>
+        </is>
+      </c>
+      <c r="H2" s="51" t="inlineStr">
+        <is>
+          <t>Bonne reponse (le numero)</t>
+        </is>
+      </c>
+      <c r="I2" s="51" t="inlineStr">
+        <is>
+          <t>Indice gagne</t>
+        </is>
+      </c>
+      <c r="J2" s="51" t="inlineStr">
+        <is>
+          <t>Message si faux</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>au scan</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>Sous son épais pelage blanc, de quelle couleur est la peau de l'ours polaire ?</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>Rose</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>Blanche</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>Noire</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>Grise</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" s="52" t="inlineStr">
+        <is>
+          <t>Félicitations ! Voici votre indice : le Talkie Walkie des soigneurs est branché sur un circuit fermé, seuls les membres de l'équipe du zoo peuvent l'utiliser.</t>
+        </is>
+      </c>
+      <c r="J3" s="52" t="inlineStr">
+        <is>
+          <t>Mauvaise réponse. Ne vous inquiétez pas, d'autres questions surprises vous seront proposées plus tard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>au scan</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>Dans une meute de loups du Canada, qui décide du moment de la chasse ?</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>Le loup le plus fort</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>Le couple de parents</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Le plus vieux loup</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="inlineStr">
+        <is>
+          <t>Chacun à tour de rôle</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="52" t="inlineStr">
+        <is>
+          <t>Félicitations ! Voici votre indice : Un intrus s'est introduit dans le Parc Zoologique &amp; Botanique cette nuit et peut semer la zizanie dans votre enquête.</t>
+        </is>
+      </c>
+      <c r="J4" s="52" t="inlineStr">
+        <is>
+          <t>Mauvaise réponse. Ne vous inquiétez pas, d'autres questions surprises vous seront proposées plus tard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>avant la sortie</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>Pourquoi des industriels mulhousiens ont-ils créé ce parc en 1868 ?</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>Pour offrir un lieu de détente à leurs ouvriers</t>
+        </is>
+      </c>
+      <c r="E5" s="52" t="inlineStr">
+        <is>
+          <t>Pour recueillir les animaux d'un cirque en faillite</t>
+        </is>
+      </c>
+      <c r="F5" s="52" t="inlineStr">
+        <is>
+          <t>Pour y élever des animaux de ferme</t>
+        </is>
+      </c>
+      <c r="G5" s="52" t="inlineStr">
+        <is>
+          <t>Pour en faire une réserve de chasse</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="52" t="inlineStr">
+        <is>
+          <t>Félicitations ! Voici votre indice : Cet interrogatoire était un peu suspect, n'est-ce pas ? Je me demande si Greg est digne de confiance.</t>
+        </is>
+      </c>
+      <c r="J5" s="52" t="inlineStr">
+        <is>
+          <t>Mauvaise réponse. Ne vous inquiétez pas, d'autres questions surprises vous seront proposées plus tard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>avant la sortie</t>
+        </is>
+      </c>
+      <c r="C6" s="52" t="inlineStr">
+        <is>
+          <t>Pourquoi des industriels mulhousiens ont-ils créé ce parc en 1868 ?</t>
+        </is>
+      </c>
+      <c r="D6" s="52" t="inlineStr">
+        <is>
+          <t>Pour offrir un lieu de détente à leurs ouvriers</t>
+        </is>
+      </c>
+      <c r="E6" s="52" t="inlineStr">
+        <is>
+          <t>Pour recueillir les animaux d'un cirque en faillite</t>
+        </is>
+      </c>
+      <c r="F6" s="52" t="inlineStr">
+        <is>
+          <t>Pour y élever des animaux de ferme</t>
+        </is>
+      </c>
+      <c r="G6" s="52" t="inlineStr">
+        <is>
+          <t>Pour en faire une réserve de chasse</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="52" t="inlineStr">
+        <is>
+          <t>Félicitations ! Voici votre indice : Cet interrogatoire était un peu suspect, n'est-ce pas ? Je me demande si Greg est digne de confiance.</t>
+        </is>
+      </c>
+      <c r="J6" s="52" t="inlineStr">
+        <is>
+          <t>Mauvaise réponse. Ne vous inquiétez pas, d'autres questions surprises vous seront proposées plus tard.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Des consignes de trajet plus précises autour des ours et des loups
Le bureau des soigneurs est situé « à côté des ours polaires », la borne
de l'enclos « en haut », et celle de la passante « au fond de
l'impasse ». Les deux sens reçoivent la précision là où ils font le même
trajet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lw9eyzA4F2s1Quh6QtCwXf
</commit_message>
<xml_diff>
--- a/contenu/sanctuaire-cahier-de-contenu.xlsx
+++ b/contenu/sanctuaire-cahier-de-contenu.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="520" windowWidth="28800" windowHeight="15900" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Parcours" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Textes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Quiz" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Pop quiz" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Denouements" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parcours" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quiz" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pop quiz" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Denouements" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="F10" s="38" t="inlineStr">
         <is>
-          <t>Rendez-vous au bureau des soigneurs pour interroger votre premier témoin.</t>
+          <t>Rendez-vous au bureau des soigneurs, à côté des ours polaires, pour interroger votre premier témoin.</t>
         </is>
       </c>
       <c r="G10" s="37" t="n"/>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="F16" s="40" t="inlineStr">
         <is>
-          <t>Rendez-vous au niveau de l'enclos des loups pour la suite de l'enquête</t>
+          <t>Rendez-vous au niveau du haut de l'enclos des loups pour la suite de l'enquête</t>
         </is>
       </c>
       <c r="G16" s="40" t="n"/>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="F20" s="37" t="inlineStr">
         <is>
-          <t>Rendez-vous au niveau de l'enclos des loups pour la suite de l'enquête</t>
+          <t>Rendez-vous au niveau du haut de l'enclos des loups pour la suite de l'enquête</t>
         </is>
       </c>
       <c r="G20" s="37" t="n"/>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="F23" s="38" t="inlineStr">
         <is>
-          <t>Rendez-vous au-dessus de l'enclos des loups pour interroger votre prochain témoin</t>
+          <t>Rendez-vous au fond de l'impasse, au-dessus de l'enclos des loups, pour interroger votre prochain témoin</t>
         </is>
       </c>
       <c r="G23" s="37" t="n"/>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="F24" s="45" t="inlineStr">
         <is>
-          <t>Rendez-vous au-dessus de l'enclos des loups pour interroger votre prochain témoin</t>
+          <t>Rendez-vous au fond de l'impasse, au-dessus de l'enclos des loups, pour interroger votre prochain témoin</t>
         </is>
       </c>
       <c r="G24" s="43" t="n"/>

</xml_diff>

<commit_message>
Le quiz animalier recalibré : six questions, la lettre après « Suivant »
La vidéo a été raccourcie. Six questions restent, à leurs nouveaux
temps : le coq (0:26), l'homme qui râle (0:45), l'alligator (1:20), le
manchot (2:13), le renard (3:13) et le zèbre (3:57). Le fou rire et le
ronfleur sont retirés du cahier. La version courte est servie sous un
nom neuf, quiz-animalier-2-hwqbca.mp4.

La lettre I quitte l'écran du quiz pour un écran à elle, après
« Suivant ». Elle arrive ainsi quel que soit le score, que la vidéo se
soit chargée ou non, et que le groupe l'ait regardée ou passée.

« Passer la vidéo », demandé sur le terrain : le bouton du quiz est
visible dès le départ sous ce nom, et devient « Suivant » à la fin.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lw9eyzA4F2s1Quh6QtCwXf
</commit_message>
<xml_diff>
--- a/contenu/sanctuaire-cahier-de-contenu.xlsx
+++ b/contenu/sanctuaire-cahier-de-contenu.xlsx
@@ -4030,7 +4030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0:35</t>
+          <t>0:26</t>
         </is>
       </c>
       <c r="C3" s="52" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0:54</t>
+          <t>0:45</t>
         </is>
       </c>
       <c r="C4" s="52" t="inlineStr">
@@ -4180,7 +4180,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1:13</t>
+          <t>1:20</t>
         </is>
       </c>
       <c r="C5" s="52" t="inlineStr">
@@ -4190,26 +4190,26 @@
       </c>
       <c r="D5" s="52" t="inlineStr">
         <is>
-          <t>Frédéric, 54 ans, qui part en fou rire</t>
+          <t>Une porte qui grince</t>
         </is>
       </c>
       <c r="E5" s="52" t="inlineStr">
         <is>
-          <t>Un dindon qui glousse</t>
+          <t>Un alligator</t>
         </is>
       </c>
       <c r="F5" s="52" t="inlineStr">
         <is>
-          <t>Un singe</t>
+          <t>Un marteau-piqueur</t>
         </is>
       </c>
       <c r="G5" s="52" t="inlineStr">
         <is>
-          <t>Une personne qui s'esclaffe</t>
+          <t>Une otarie</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1:39</t>
+          <t>2:13</t>
         </is>
       </c>
       <c r="C6" s="52" t="inlineStr">
@@ -4230,26 +4230,26 @@
       </c>
       <c r="D6" s="52" t="inlineStr">
         <is>
-          <t>Chewbacca</t>
+          <t>C'est de la techno !</t>
         </is>
       </c>
       <c r="E6" s="52" t="inlineStr">
         <is>
-          <t>Un rhinocéros</t>
+          <t>Un vautour</t>
         </is>
       </c>
       <c r="F6" s="52" t="inlineStr">
         <is>
-          <t>Une personne qui ronfle</t>
+          <t>Un flamant rose</t>
         </is>
       </c>
       <c r="G6" s="52" t="inlineStr">
         <is>
-          <t>Un tigre</t>
+          <t>Un manchot</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2:03</t>
+          <t>3:13</t>
         </is>
       </c>
       <c r="C7" s="52" t="inlineStr">
@@ -4270,22 +4270,22 @@
       </c>
       <c r="D7" s="52" t="inlineStr">
         <is>
-          <t>Une porte qui grince</t>
+          <t>Une femme qui crie de détresse</t>
         </is>
       </c>
       <c r="E7" s="52" t="inlineStr">
         <is>
-          <t>Un alligator</t>
+          <t>Un renard</t>
         </is>
       </c>
       <c r="F7" s="52" t="inlineStr">
         <is>
-          <t>Un marteau-piqueur</t>
+          <t>Une souricette</t>
         </is>
       </c>
       <c r="G7" s="52" t="inlineStr">
         <is>
-          <t>Une otarie</t>
+          <t>Un corbeau</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2:58</t>
+          <t>3:57</t>
         </is>
       </c>
       <c r="C8" s="52" t="inlineStr">
@@ -4310,108 +4310,30 @@
       </c>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t>C'est de la techno !</t>
+          <t>Un zèbre</t>
         </is>
       </c>
       <c r="E8" s="52" t="inlineStr">
         <is>
-          <t>Un vautour</t>
+          <t>Un gecko</t>
         </is>
       </c>
       <c r="F8" s="52" t="inlineStr">
         <is>
-          <t>Un flamant rose</t>
+          <t>Une alarme de voiture de police</t>
         </is>
       </c>
       <c r="G8" s="52" t="inlineStr">
         <is>
-          <t>Un manchot</t>
+          <t>Une sonnerie de téléphone</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>E06</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>3:59</t>
-        </is>
-      </c>
-      <c r="C9" s="52" t="inlineStr">
-        <is>
-          <t>Bruit d'humain ou d'animal ?</t>
-        </is>
-      </c>
-      <c r="D9" s="52" t="inlineStr">
-        <is>
-          <t>Une femme qui crie de détresse</t>
-        </is>
-      </c>
-      <c r="E9" s="52" t="inlineStr">
-        <is>
-          <t>Un renard</t>
-        </is>
-      </c>
-      <c r="F9" s="52" t="inlineStr">
-        <is>
-          <t>Une souricette</t>
-        </is>
-      </c>
-      <c r="G9" s="52" t="inlineStr">
-        <is>
-          <t>Un corbeau</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>E06</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>4:42</t>
-        </is>
-      </c>
-      <c r="C10" s="52" t="inlineStr">
-        <is>
-          <t>Bruit d'humain ou d'animal ?</t>
-        </is>
-      </c>
-      <c r="D10" s="52" t="inlineStr">
-        <is>
-          <t>Un zèbre</t>
-        </is>
-      </c>
-      <c r="E10" s="52" t="inlineStr">
-        <is>
-          <t>Un gecko</t>
-        </is>
-      </c>
-      <c r="F10" s="52" t="inlineStr">
-        <is>
-          <t>Une alarme de voiture de police</t>
-        </is>
-      </c>
-      <c r="G10" s="52" t="inlineStr">
-        <is>
-          <t>Une sonnerie de téléphone</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="9" ht="30" customHeight="1"/>
+    <row r="10" ht="30" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
La fin de la serre : la vidéo, puis l'aveu de Greg, puis le mot de la fin
Après les conclusions, la vidéo de la serre reçoit un bouton « Suivant ».
Vient ensuite un écran pour la photo de l'aveu de Greg
(assets/img/aveu-greg.webp, à déposer), puis l'écran de fin : « L'affaire
est classée. », les remerciements et les partenaires.

La ligne « 5. Finish », restée vide dans le cahier, devient l'écran de la
photo ; une ligne « 6. Fin » est ajoutée.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lw9eyzA4F2s1Quh6QtCwXf
</commit_message>
<xml_diff>
--- a/contenu/sanctuaire-cahier-de-contenu.xlsx
+++ b/contenu/sanctuaire-cahier-de-contenu.xlsx
@@ -1696,7 +1696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3909,20 +3909,20 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>5. Finish</t>
+          <t>5. Photo : l'aveu de Greg</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Message final à délivrer en fonction des conclusions du groupe dans le champs IA</t>
-        </is>
-      </c>
-      <c r="F68" s="12" t="n"/>
-      <c r="G68" s="12" t="inlineStr">
-        <is>
-          <t>3 messages de félicitations (parfait - presque - dommage)</t>
-        </is>
-      </c>
+          <t>La legende sous la photo de l'aveu. Une ligne.</t>
+        </is>
+      </c>
+      <c r="F68" s="12" t="inlineStr">
+        <is>
+          <t>Une dernière pièce au dossier : l'aveu de Greg.</t>
+        </is>
+      </c>
+      <c r="G68" s="12" t="n"/>
     </row>
     <row r="69" ht="30" customFormat="1" customHeight="1" s="39">
       <c r="A69" s="34" t="inlineStr">
@@ -4018,6 +4018,38 @@
         </is>
       </c>
       <c r="G71" s="37" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>E15</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>La serre</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>les deux</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>6. Fin</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Le mot de la fin, au-dessus des remerciements et des partenaires.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>L'affaire est classée.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Les quatre images du commissaire, après son appel
Après l'appel, un écran annonce « Le commissaire vous a envoyé 4
images. » et ouvre un carrousel (commissaire-1.webp à commissaire-4.webp,
à déposer dans assets/img/). La ligne 54 du cahier, restée vide, porte
désormais ce texte.

Les carrousels deviennent réglables (écran, texte du bouton, photos), et
leur texte passe au-dessus du bouton qu'il annonce, au sac du botaniste
aussi. Leurs boutons deviennent « ‹ Précédente » et « Suivante › » : un
« Suivant » de plus se confondait avec celui qui quitte l'écran.

L'aveu de Greg passe de 1,5 Mo à 79 Ko (1080 px de large), pour la 4G du
parc.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lw9eyzA4F2s1Quh6QtCwXf
</commit_message>
<xml_diff>
--- a/contenu/sanctuaire-cahier-de-contenu.xlsx
+++ b/contenu/sanctuaire-cahier-de-contenu.xlsx
@@ -3435,7 +3435,7 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>3. Texte ou epreuve</t>
+          <t>3. Les images du commissaire</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
@@ -3445,14 +3445,10 @@
       </c>
       <c r="F54" s="12" t="inlineStr">
         <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="G54" s="12" t="inlineStr">
-        <is>
-          <t>Fichier audio</t>
-        </is>
-      </c>
+          <t>Le commissaire vous a envoyé 4 images.</t>
+        </is>
+      </c>
+      <c r="G54" s="12" t="n"/>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="37" t="inlineStr">

</xml_diff>

<commit_message>
La fin à la serre : un choix parmi quatre, la vérité, puis le verdict
L'IA départageait mal les conclusions écrites : on la débranche.

- Les conclusions deviennent un choix parmi quatre propositions. Le choix
  mène droit à la vidéo de la serre, sans dire au groupe s'il a raison.
- Puis la lettre de Greg (plus « l'aveu »), puis le verdict : étincelles
  et félicitations pour la bonne réponse, dénouement « Mauvais » sinon.
- Le photocall a son propre écran, entre le verdict et les remerciements.
- Le choix est verrouillé : revenir en arrière après la vidéo ne permet
  pas de le changer. Il est toujours rangé dans la base pour le tableau
  de bord.
- Le juge par IA et par mots-clés est retiré, ainsi que la fonction
  Supabase juger-conclusions et sa notice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lw9eyzA4F2s1Quh6QtCwXf
</commit_message>
<xml_diff>
--- a/contenu/sanctuaire-cahier-de-contenu.xlsx
+++ b/contenu/sanctuaire-cahier-de-contenu.xlsx
@@ -3845,12 +3845,12 @@
       </c>
       <c r="F66" s="12" t="inlineStr">
         <is>
-          <t>Veuillez nous donner les conclusions de votr enquête. Qu'est arrivé à Isabelle ?</t>
+          <t>Qu'est-il arrivé à Isabelle ?</t>
         </is>
       </c>
       <c r="G66" s="12" t="inlineStr">
         <is>
-          <t>Champ IA pour donner ses conclusions</t>
+          <t>Choix multiple : les quatre propositions sont dans CONCLUSIONS_QCM (fabriquer-les-pages.py)</t>
         </is>
       </c>
     </row>
@@ -3905,17 +3905,17 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>5. Photo : l'aveu de Greg</t>
+          <t>5. Photo : la lettre de Greg</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>La legende sous la photo de l'aveu. Une ligne.</t>
+          <t>La legende sous la photo de la lettre. Une ligne.</t>
         </is>
       </c>
       <c r="F68" s="12" t="inlineStr">
         <is>
-          <t>Une dernière pièce au dossier : l'aveu de Greg.</t>
+          <t>Une dernière pièce au dossier : la lettre de Greg.</t>
         </is>
       </c>
       <c r="G68" s="12" t="n"/>

</xml_diff>

<commit_message>
Plus de chrono de 3 h : la partie vaut jusqu'à minuit, et s'éteint 30 minutes après la réponse finale
Les groupes visitent le zoo en même temps qu'ils jouent, et beaucoup
étaient coupés avant la fin.

- Correctif 13 : activer_code fixe la fin à minuit (heure de Paris) le
  jour de l'activation ; enregistrer_conclusions éteint le code 30 minutes
  après la réponse finale ; les parties du jour coupées sans conclusions
  sont rouvertes jusqu'à minuit.
- Chaque borne redemande l'heure de fin à la base (reprendre_partie) :
  une prolongation ou une fin de partie s'applique au prochain scan. Base
  muette : on ne coupe personne.
- Plus de compte à rebours à l'écran ; textes d'accueil et de fin revus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lw9eyzA4F2s1Quh6QtCwXf
</commit_message>
<xml_diff>
--- a/contenu/sanctuaire-cahier-de-contenu.xlsx
+++ b/contenu/sanctuaire-cahier-de-contenu.xlsx
@@ -1775,12 +1775,12 @@
       </c>
       <c r="E3" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Une page de texte avec le chrono qui se lance, le logo du jeu et une photo d'arrière plan. </t>
+          <t xml:space="preserve">Une page de texte le logo du jeu et une photo d'arrière plan. </t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>Bienvenue au Parc Zoologique &amp; Botanique de Mulhouse. Vous êtes sur le point de prendre part à une expérience unique en son genre : une enquête de police grandeur nature. Armez-vous de bon sens et observez bien ce qu'il se passe autour de vous. Suivez les consignes qui vous sont données et respectez le sens des énigmes qui vous est proposé. Vous avez 3 heures à partir de maintenant pour terminer l'enquête. Cliquez sur suivant pour démarrer votre enquête.</t>
+          <t>Bienvenue au Parc Zoologique &amp; Botanique de Mulhouse. Vous êtes sur le point de prendre part à une expérience unique en son genre : une enquête de police grandeur nature. Armez-vous de bon sens et observez bien ce qu'il se passe autour de vous. Suivez les consignes qui vous sont données et respectez le sens des énigmes qui vous est proposé. Prenez votre temps : votre enquête reste ouverte jusqu'à la fin de la journée. Cliquez sur suivant pour démarrer votre enquête.</t>
         </is>
       </c>
       <c r="G3" s="29" t="n"/>

</xml_diff>